<commit_message>
Fix financial health ratio calculations
</commit_message>
<xml_diff>
--- a/data/synthetic_history/recovery_2026/reports/university_financial_report_2026_01.xlsx
+++ b/data/synthetic_history/recovery_2026/reports/university_financial_report_2026_01.xlsx
@@ -12,12 +12,14 @@
     <sheet name="Expenses" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Budget_vs_Actual" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Department_Summary" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Payroll" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Student_Payments" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Cash_Flow" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Scholarships" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Vendor_Payments" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Anomalies_Embedded" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Financial_Position" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Payroll" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Student_Payments" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Cash_Flow" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Scholarships" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Vendor_Payments" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Anomalies_Embedded" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Goals_Targets" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -26,8 +28,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -67,12 +70,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -695,6 +699,309 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="19" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Scholarships - January 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Small/medium university | Synthetic recovery history</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Currency: USD | Synthetic data | Generated deterministically</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Period</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Month</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Department</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Scholarship_Type</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Allocated</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Awarded</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Remaining</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Recipients</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>Utilization_Pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="n">
+        <v>46023</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>January</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Need-based</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>27442.8</v>
+      </c>
+      <c r="F6" t="n">
+        <v>25410</v>
+      </c>
+      <c r="G6" t="n">
+        <v>2032.8</v>
+      </c>
+      <c r="H6" t="n">
+        <v>48</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.9258999999999999</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="n">
+        <v>46023</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>January</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Need-based</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>24948</v>
+      </c>
+      <c r="F7" t="n">
+        <v>23100</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1848</v>
+      </c>
+      <c r="H7" t="n">
+        <v>44</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.9258999999999999</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="n">
+        <v>46023</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>January</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Health Sciences</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Need-based</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>32432.4</v>
+      </c>
+      <c r="F8" t="n">
+        <v>30030</v>
+      </c>
+      <c r="G8" t="n">
+        <v>2402.4</v>
+      </c>
+      <c r="H8" t="n">
+        <v>57</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.9258999999999999</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="n">
+        <v>46023</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>January</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Arts &amp; Humanities</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Need-based</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>17463.6</v>
+      </c>
+      <c r="F9" t="n">
+        <v>16170</v>
+      </c>
+      <c r="G9" t="n">
+        <v>1293.6</v>
+      </c>
+      <c r="H9" t="n">
+        <v>31</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.9258999999999999</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="n">
+        <v>46023</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>January</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Student Services</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Need-based</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>12474</v>
+      </c>
+      <c r="F10" t="n">
+        <v>11550</v>
+      </c>
+      <c r="G10" t="n">
+        <v>924</v>
+      </c>
+      <c r="H10" t="n">
+        <v>22</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.9258999999999999</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="n">
+        <v>46023</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>January</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Administration</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Need-based</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>9979.200000000001</v>
+      </c>
+      <c r="F11" t="n">
+        <v>9240</v>
+      </c>
+      <c r="G11" t="n">
+        <v>739.2</v>
+      </c>
+      <c r="H11" t="n">
+        <v>18</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.9258999999999999</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1124,7 +1431,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1161,6 +1468,245 @@
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>No_Data</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Goals Targets - January 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Small/medium university | Synthetic recovery history</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Currency: USD | Synthetic data | Generated deterministically</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Period</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Goal_ID</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Meta</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Target_Value</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Actual_Value</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026_01</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>GOAL-OPERATING-MARGIN</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Mantener resultado operativo positivo</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>net_operating_result</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>82500</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>cumple</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026_01</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>GOAL-PAYROLL-RATIO</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Mantener la relación nómina/ingresos en 42% o menos</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>payroll_percentage_of_revenue</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>ratio</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>cumple</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026_01</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>GOAL-COLLECTION-RATE</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Alcanzar una tasa de cobranza de al menos 94%</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>collection_rate</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>ratio</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>cumple</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026_01</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>GOAL-CASH-FLOW</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Evitar flujo neto de caja negativo</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>net_cash_flow</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
+        <v>150000</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>cumple</t>
         </is>
       </c>
     </row>
@@ -3755,6 +4301,130 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Financial Position - January 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Small/medium university | Synthetic recovery history</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Currency: USD | Synthetic data | Generated deterministically</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Period</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Month</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Current_Assets</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Current_Liabilities</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Cash_and_Equivalents</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Total_Assets</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Total_Liabilities</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>EBITDA</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>Net_Income</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="n">
+        <v>46023</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>January</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>3922000</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1762500</v>
+      </c>
+      <c r="E6" t="n">
+        <v>2650000</v>
+      </c>
+      <c r="F6" t="n">
+        <v>10357000</v>
+      </c>
+      <c r="G6" t="n">
+        <v>4770500</v>
+      </c>
+      <c r="H6" t="n">
+        <v>647400</v>
+      </c>
+      <c r="I6" t="n">
+        <v>37500</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -4088,7 +4758,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5273,7 +5943,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5458,307 +6128,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:I11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="19" customWidth="1" min="9" max="9"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Scholarships - January 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Small/medium university | Synthetic recovery history</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Currency: USD | Synthetic data | Generated deterministically</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Period</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Month</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Department</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>Scholarship_Type</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>Allocated</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>Awarded</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>Remaining</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>Recipients</t>
-        </is>
-      </c>
-      <c r="I5" s="3" t="inlineStr">
-        <is>
-          <t>Utilization_Pct</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="n">
-        <v>46023</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>January</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Engineering</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Need-based</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>27442.8</v>
-      </c>
-      <c r="F6" t="n">
-        <v>25410</v>
-      </c>
-      <c r="G6" t="n">
-        <v>2032.8</v>
-      </c>
-      <c r="H6" t="n">
-        <v>48</v>
-      </c>
-      <c r="I6" t="n">
-        <v>0.9258999999999999</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="n">
-        <v>46023</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>January</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Business</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Need-based</t>
-        </is>
-      </c>
-      <c r="E7" t="n">
-        <v>24948</v>
-      </c>
-      <c r="F7" t="n">
-        <v>23100</v>
-      </c>
-      <c r="G7" t="n">
-        <v>1848</v>
-      </c>
-      <c r="H7" t="n">
-        <v>44</v>
-      </c>
-      <c r="I7" t="n">
-        <v>0.9258999999999999</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="n">
-        <v>46023</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>January</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Health Sciences</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Need-based</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>32432.4</v>
-      </c>
-      <c r="F8" t="n">
-        <v>30030</v>
-      </c>
-      <c r="G8" t="n">
-        <v>2402.4</v>
-      </c>
-      <c r="H8" t="n">
-        <v>57</v>
-      </c>
-      <c r="I8" t="n">
-        <v>0.9258999999999999</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="n">
-        <v>46023</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>January</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Arts &amp; Humanities</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Need-based</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>17463.6</v>
-      </c>
-      <c r="F9" t="n">
-        <v>16170</v>
-      </c>
-      <c r="G9" t="n">
-        <v>1293.6</v>
-      </c>
-      <c r="H9" t="n">
-        <v>31</v>
-      </c>
-      <c r="I9" t="n">
-        <v>0.9258999999999999</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="n">
-        <v>46023</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>January</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Student Services</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Need-based</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>12474</v>
-      </c>
-      <c r="F10" t="n">
-        <v>11550</v>
-      </c>
-      <c r="G10" t="n">
-        <v>924</v>
-      </c>
-      <c r="H10" t="n">
-        <v>22</v>
-      </c>
-      <c r="I10" t="n">
-        <v>0.9258999999999999</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="n">
-        <v>46023</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>January</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Administration</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Need-based</t>
-        </is>
-      </c>
-      <c r="E11" t="n">
-        <v>9979.200000000001</v>
-      </c>
-      <c r="F11" t="n">
-        <v>9240</v>
-      </c>
-      <c r="G11" t="n">
-        <v>739.2</v>
-      </c>
-      <c r="H11" t="n">
-        <v>18</v>
-      </c>
-      <c r="I11" t="n">
-        <v>0.9258999999999999</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>